<commit_message>
Build-45 payload complete: Spending tab conforms to the approved mock (row 40 closed) + income pop-up v2 FINAL mock + design changelog + the founder's launch sign-off sheet
Spending: month header with the sum, recent rows with Teller-ready source
chips, categories-vs-plan, All-transactions + Import doors opening the
proven full bodies, day-one three doors. 2 new pins; 1258 green.
Launch sign-off: docs/FCC-core-55-70/launch-signoff-v1-2026-07-19.xlsx —
40 screens, verdict dropdown (READY FOR LAUNCH / FEEDBACK) + feedback column.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2955,6 +2955,60 @@
       <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Founder — APPROVED 2026-07-19 ("cashflow. Approve.")</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Cash flow</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Income pop-up (v2): "Which 12 months are you entering?" — Calendar year N or Next 12 months; every month chip and editor carries month + year (incl. across the New-Year boundary); both frames write the same canonical calendar slots; note "this yearly pattern repeats". Receipt scanning: totals never read from payment-mechanics lines.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Founder Build-44 findings (rows 33-34)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Founder — directed 2026-07-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Cash flow</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Spending tab conformance: month header with the sum, recent rows with source chips (by hand / imported; bank arrives with Teller), categories-vs-plan card, All-transactions and Import doors opening the proven full bodies; day-one three doors.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Founder Build-44 finding (row 40) — conform to the approved mock</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Approved mock is the spec</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Founder decision round 2026-07-28: 10 audit decisions logged + Build-46 item walk delivered
- build46-item-walk-v1-2026-07-28.xlsx: 16 fixes, one row each (today -> after,
  exact copy, mock status), APPROVE/CHANGE/SKIP dropdown — founder walks per row
- design v1.3 Changelog +7 rows: Sample gauge wins empty-odds, disconnect =
  offer-the-choice, cushion card reinstated (mock first), type-size question
  CLOSED (tables keep approved sizes), legacy modules STAY in v1, validated
  colorblind palettes to be adopted (recolored mocks first), same-day-changelog
  rule adopted
- CLAUDE.md: SAME-DAY CHANGELOG standing order
- build-analysis-july24.xlsx: byte-identical content, Excel re-save on open

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3009,6 +3009,195 @@
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Approved mock is the spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Empty-state odds strip RESOLVED: the locked Sample gauge ("Sample: 84% to age 92") is the approved empty state. The later 3-questions-invite mock is retired.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Two approvals conflicted by date (Jul-15 gauge vs later mock); the July-24 audit surfaced it; founder picked the gauge.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Founder — DECIDED 2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Net worth / Connect / Settings</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Disconnect promise UNIFIED: on disconnect the user is offered the choice — keep the numbers as a by-hand account, or delete the connection’s data. Consent copy, Settings, and the future account-page door all state this same promise. Exact copy rides the Build-46 item walk for approval.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Doc said "numbers stay", shipped consent said "we delete" — behavior in Settings already offered the choice; founder aligned the promise to the choice.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Founder — DECIDED 2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Net worth</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Emergency-cushion card ("X months of essentials", below the fold) REINSTATED as to-build: it returns to scope, mock first — founder approves the drawn Net worth screen before any code.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Doc specified it; v7 FINAL mock dropped it; the July-24 audit put the drop-or-build call to the founder, who chose build.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Founder — DECIDED 2026-07-28 (build after mock approval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>All screens</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Type-size question CLOSED: dense tables (Invest winners/laggards, holdings list) keep their approved compact sizes; the 17-point money floor applies to heroes and standalone money only.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Long-open decision (17pt floor vs dense tables); the approved v7 tables set the precedent; founder confirmed.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Founder — DECIDED 2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Screen inventory</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Legacy modules (Estate, Insurance, Tax organizer, Job safety, Credit) STAY in the v1 launch. They remain rows in the 97-row launch sign-off walk and must each pass it.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Not covered by FCC docs; audit asked keep-vs-hide; founder chose keep for launch value.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Founder — DECIDED 2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>All screens</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Chart colors: the UX doc’s validated colorblind-safe palettes WILL BE ADOPTED app-wide (one consistent set; e.g. Cash gets one color everywhere). Recolored mocks of every affected chart come first; nothing changes until the founder approves the pictures.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Shipped colors drifted between screens and the validated palettes were never adopted; colorblind-safe is a stated UX standard.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Founder — DECIDED 2026-07-28 (adopt after mock approval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>STANDING RULE ADOPTED: every founder approval gets a dated row in this Changelog tab the same day, alongside the mock. Also recorded in the repo’s CLAUDE.md.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Root cause of doc-vs-code drift found by the July-24 audit: dozens of July approvals, 4 changelog rows.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Founder — ADOPTED 2026-07-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build-47 walk 25/25 BUILT: master file (27 cells + findings + plan) → BUILT, walk outcomes col J, same-day changelog row — suite 1,311 green, tsc clean
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3252,6 +3252,33 @@
       <c r="E14" t="inlineStr">
         <is>
           <t>Doc correction — evidence in git history</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>All screens</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BUILD-47 WALK BUILT — all 25 rows approved verbally ("Approve all 25") and coded with pins: HSA honest cap · SS claim-NOW at 68-69 · RMD card taken-check · value-as-of in bond/alt editors · undated-value nudge · rothConversionCost canonical · capacity derived from surplusByMonth · sourceWording shared · RMD schedule on the shared growth step · snapshot reads blendedReturn · HeroAmount (5 heroes) · hidden-balances banner ×5 tabs · pull-to-refresh · approved door lines · Roth banner+save+dated hub to-do · period sync · tappable concentration · double-fire suppression · possible_duplicate flag (incl. manual) · Reduce Motion ×19 modal files · component spoken label · shared picker naming · confirm-before-remove · plain income note+door · add-any-income-source. Plus B46 findings 7/8/10 accuracy fixes. Suite 1,289 → 1,311.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Founder approval 2026-07-30 (Build-47 walk, all rows)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Founder — APPROVED 2026-07-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Palettes ADOPTED (founder YES): validated fixed-order set into ChartPalette/ClassMarkColors + successGreen good-mark; exact values pinned; mock → final; changelog + master cells
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3279,6 +3279,33 @@
       <c r="E15" t="inlineStr">
         <is>
           <t>Founder — APPROVED 2026-07-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>All screens</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>VALIDATED COLOR PALETTES ADOPTED (founder YES on chart-palettes-v2 FINAL): ChartPalette + ClassMarkColors moved to the UX doc's colorblind-validated fixed-order set (#2a78d6 stocks · #1baf7a cash · #eda100 real estate · #4a3aa7 bonds · #eb6834 alternatives · #e87ba4 personal · #898781 mixed); successGreen marks → the validated good step #0ca30c. Colors ONLY — layouts/words/numbers unchanged per the mock's stated rule. Exact values pinned by test.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>UX doc Color tab (validated set was specified, never adopted); founder approval 2026-07-30</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Founder — APPROVED 2026-07-30 ("yes")</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Staleness stamps BUILT (mock 4 approved + founder's left-justified change): in-hero amber stamp on Home + NW when a connection is 3+ days stale; standalone line → retired lens only; stale/fresh pins; v2 as-built mock → final
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3306,6 +3306,33 @@
       <c r="E16" t="inlineStr">
         <is>
           <t>Founder — APPROVED 2026-07-30 ("yes")</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Home · Net worth</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>STALENESS STAMPS BUILT (mock #4 approved with founder change): when a connected account is 3+ days old, the Home hero and Net worth hero carry one amber line inside the box — "⏱ &lt;institution&gt; part as of &lt;date&gt; — N days old · pull to refresh" — left-justified like their sibling lines. The standalone stale line now serves the retired lens only (its hero has no investments box).</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Founder approval 2026-07-31 with the left-justified change; mock v2 = as-built record</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Founder — APPROVED 2026-07-31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mock-verdict round BUILT: dark separator dots (pick C, Colors.sepDot + DotJoined), source chips, cushion card (3 states), matured-bond banner (ledger-wired), add/record router (real editors, separate fields), path-ahead how-i; 1,319 green, tsc clean
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3331,6 +3331,33 @@
         </is>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>Founder — APPROVED 2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NW · Invest · Home · app-wide</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MOCK-BATCH VERDICT ROUND BUILT: separator dots = the DARKER designed glyph (founder pick C — visibility for 55-70 eyes; Colors.sepDot token + DotJoined on marquee lines) · source chips on NW rows (approved) · cushion card (approved; 3 states) · matured-bond banner (approved; paid-out writes the ledger) · add/record ROUTER (findings 3+6; chips open the real editors with separate fields, Record gains bond/alt doors) · path-ahead row stays its own card + gains the how-ⓘ (nestEggMath) · "See your growth" KEPT as-is · staleness stamps in-hero, left-justified · sentence periods stay (founder call). Suite 1,319 green.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Founder verdicts 2026-07-31 in chat</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Founder — APPROVED 2026-07-31</t>
         </is>

</xml_diff>

<commit_message>
Loading/offline pins + records: 1,321 green; master cells + changelog current
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3358,6 +3358,33 @@
         </is>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>Founder — APPROVED 2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Home · app root · Invest sheets</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>LOADING/OFFLINE DECIDED+BUILT: couldn't-refresh banner on Home (store-flagged, honest as-of, clears on success); the mock's grey-bar skeleton REJECTED by founder question and replaced by the root hydration hold (no screen renders before the store is ready — sub-second, kills the cold-start doors-flash). Router mock v2 delivered per founder revision (drawn from the shipping editors, separate fields).</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Founder verdicts 2026-07-31</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Founder — APPROVED 2026-07-31</t>
         </is>

</xml_diff>

<commit_message>
B47 findings 1-2 FIXED: equity symbol field (live-price row seeding) + bottom Done on the editor modal; Build 47 findings tab created; pins green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3387,6 +3387,33 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>Founder — APPROVED 2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Income (equity editor)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>B47 WALK FINDINGS 1-2 FIXED: equity editor gains the company stock symbol field (live price seeds new rows, editable; full re-marking joins the provider work) and a real bottom Done button (the top-bar link was invisible from a long form; "saves as you type" note).</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Founder Build-47 walk findings, 2026-07-31</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Founder findings — fixed same hour</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 finding 3 (Vanguard): balance derives from holdings when the broker total is missing/zero — USD-gated, empty-stays-zero, authority intact; 3 ingest pins; findings tab + changelog
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3414,6 +3414,33 @@
       <c r="E20" t="inlineStr">
         <is>
           <t>Founder findings — fixed same hour</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Connected accounts (ingest)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>B47 FINDING 3 FIXED (Vanguard): balance authority rule gains the derive-from-holdings fallback when the broker reports no usable total (missing/zero) — marks + options + cash sleeve; USD-only (currency guard); empty stays zero; real totals still win. 3 new ingest pins.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Founder Build-47 walk (second live institution)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Founder finding — fixed same hour</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 finding 11 (founder-approved mock): ONE repayment-shaped debt editor
- DebtEditorSheet replaces the drifted Net-worth + Cash-flow forms
- installment: real payment <-> paid-off-by, either computed (monthsToClear/paymentToClearBy)
- due_in_full: amount + date -> single dated big-ticket in grid + bill calendar + Later;
  zero monthly obligation in DTI/cash flow, balance still hits net worth, payoff plan merges it
- 20 pins across domain + walk suite; 1351 green, tsc clean

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3441,6 +3441,33 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>Founder finding — fixed same hour</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cash flow / Net worth — debts</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ONE debt editor shaped by repayment (installment: real payment ↔ paid-off-by; cards: min + you-pay; due in full: amount + date → dated big-ticket in cash flow + bill calendar). Replaces the two drifted debt forms.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>B47 walk finding 11: mortgage end year + actual payment were never asked; a loan due in full on a date was unrepresentable. Mock debt-editor-v1-2026-07-31 approved.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Founder (chat, "approved.")</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 findings 12+13: one slider drag engine (sliderGesture.ts) + honest coasting-box copy
- finding 12: cockpit's private slider had the pre-device-fix drag code (scroll steal,
  stale anchor); both sliders now ride ONE engine with capture/termination/native-block/
  pageX lessons; scenario page scroll stands down mid-drag; guard pins PanResponder.create
  to sliderGesture.ts only; cockpit sliders gain adjustable a11y
- finding 13: left box states each read as one sentence (gets there by N / doesn't, even by 80)
- 1357 green, tsc clean

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3468,6 +3468,33 @@
       <c r="E22" t="inlineStr">
         <is>
           <t>Founder (chat, "approved.")</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Retirement — Where you stand</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Coasting box copy: each state one sentence ("today's $X alone gets there by N" / "alone doesn't get there — even by 80"); "growing at %" wording</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>B47 walk finding 13: the three stacked fragments contradicted each other</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Founder (device finding; fix per plain-English rule)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 finding 6 (approved mock v2): holding screen rebuilt — price hero, graph + period chips, one table grammar
- CURRENT PRICE hero w/ prior-close change (honest stale wording), sparkline from real closes
- position/compare/lots/dividends-realized/tax as tables; compare window words match capped math
- unpriced: basis hero + provider note; maskedPrice3 keeps sub-$2 averages at 3 decimals, masked
- edit -> pencil in header; 6 pins superseded, 2 added; cashflow test clock pinned (Aug-1 flake)
- 1358 green, tsc clean

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3495,6 +3495,33 @@
       <c r="E23" t="inlineStr">
         <is>
           <t>Founder (device finding; fix per plain-English rule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Invest — holding detail</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Full page rebuilt to mock v2: price hero + graph + period chips, position/compare/lots/dividends-realized/tax all in one table grammar; ✎ edit in header; unpriced = honest basis hero with 3-decimal averages</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>B47 walk finding 6; mock holding-detail-full-v2-2026-07-31 approved</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Founder (chat, "holding screen - approved.")</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 finding 14: By-type cash group = 'Cash and cash equivalents' (one CASH_GROUP_LABEL, all cash kinds merge); row-8 pin superseded
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3522,6 +3522,33 @@
       <c r="E24" t="inlineStr">
         <is>
           <t>Founder (chat, "holding screen - approved.")</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Net worth — By type view</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>All cash-bucket account types merge under one group header "Cash and cash equivalents" (was per-type headers, e.g. "Savings" covering CD + money market + cash)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>B47 walk finding 14: founder — call it what it is</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan hub mock v9: 'Can I afford it?' (founder dropped 'all'); grammar decision logged in changelog
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3547,6 +3547,33 @@
         </is>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Plan hub (redesign in review)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Decision-row grammar: every row a complete first-person question — When can I retire? / Can I afford it? (founder dropped "all") / When should I claim Social Security? / Which account do I draw from first? / Is a Roth move worth it? / Can I spend more?</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Founder verdict on mock v8 research round ("like it"); NN/g 65+ readability + industry best practice</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
         </is>

</xml_diff>

<commit_message>
Plan hub rebuilt to approved mock v9: gauge verdicts w/ if-clause, one dated next-decision, retiree paycheck card (Home engine), dynamic door, question rows, locks, sandbox; 7 new pins + 4 superseded; big-costs capture mocked; Build-48 payload tab
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3574,6 +3574,60 @@
         </is>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Plan hub</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>FULL REDESIGN BUILT to mock v9 (founder: "all mock up approved"): spectrum gauge verdicts w/ if-clause per lens, ONE dated next-decision card (required withdrawal &gt; SS window), retiree paycheck card = Home engine, dynamic first-day door counting only missing answers + crediting accounts, question-grammar rows ranked by mind-order, honest locks, fenced sandbox</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Plan-tab redesign round, mocks v1→v9</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plan hub</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>"What big costs are coming?" feature APPROVED; capture screen mocked (big-costs-v1) — builds on its approval; hub row lands with it</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>One-time future costs invisible to the long-range odds today</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
         </is>

</xml_diff>

<commit_message>
v9 grammar sweep: ss-timing route title 'When should I claim Social Security?'; adoption sheet 'Plan to claim' (planning, not claiming); pin updated
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3628,6 +3628,33 @@
         </is>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Screen inventory</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Orphan/legacy screens (income-detail, old income/invest/savings, Tips, Rewards) KEPT — reusable when building for other age groups; menu unchanged</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Founder decision on the primary-flows document</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
         </is>

</xml_diff>

<commit_message>
Pre-48 decision round: 9 founder decisions logged (changelog) + Build-48 payload expanded
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3657,6 +3657,249 @@
       <c r="E29" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Plan / big costs</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>big-costs-v1 capture mock APPROVED — capture + simulation + hub row build into 48</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Pre-48 decision round</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>All adoption surfaces</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ONE adopt verb: "Use as my plan" everywhere (sweep same day)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Pre-48 decision round</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Invest / holding detail</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Look-back card KEPT on the holding page (mock omission was a drawing gap)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Pre-48 decision round</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Plan / Social Security</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>"Remind me" at the claim window BUILDS into 48 (existing notification scaffolding)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pre-48 decision round</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Stress test · Insights · Tips</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Advice voice SOFTENED to fact-plus-choice on all three ("set this as a goal" class removed)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Pre-48 decision round</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Menu (TopBar)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Rewards, Tips, Build-credit tiles LEAVE the 55-70 menu; College planner + Estate stay; screens all kept in code</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Pre-48 decision round</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Insights · Cash flow</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Goal-offtrack insight + "Add something else" link BUILD into 48; Invest return-breakdown goes MOCK-FIRST (next batch)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Pre-48 decision round</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SS · multi-goal · Roth</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>STEPPERS stay (65+ precision); design sheet slider rows to be refreshed to match</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Pre-48 decision round</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Paycheck card</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>4%-guideline heads-up REWORDED to own-math framing ("above what your own numbers support long-term")</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Pre-48 decision round</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Provider pivot logged: SnapTrade out, Plaid for beta (changelog + payload row 9)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3900,6 +3900,33 @@
       <c r="E38" t="inlineStr">
         <is>
           <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Connect flow (F1)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PROVIDER PIVOT: SnapTrade OUT (founder saw connected financials displayed in its dashboard — privacy call), Plaid IN for beta. Migration = next workstream AFTER Build 48 (seam absorbs it: Plaid link swap, Investments ingest mapping, consent copy, disconnect/heal). NEW design-first feature unlocked: credit-card transaction import (Transactions + Liabilities products). Founder accepts one-time reconnect cost at LLC/launch re-setup.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Founder decision (checked SnapTrade dashboard)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Provider pivot marked ON HOLD (founder evaluating Plaid/SnapTrade/Teller)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3925,6 +3925,33 @@
         </is>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Connect flow (F1)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Provider pivot ON HOLD — founder evaluating Plaid vs SnapTrade vs Teller directly; no code or stack changes meanwhile</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Founder redirect same day</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
         </is>

</xml_diff>

<commit_message>
Return breakdown BUILT to approved mock (r16): ledger-only four lines summing to the period total; 2 pins; docs logged
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4035,6 +4035,33 @@
       <c r="E43" t="inlineStr">
         <is>
           <t>Recorded by audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Invest</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Return breakdown BUILT to approved mock (Price change · Realized · Dividends · Interest under the period total; sparse-honest; ledger-only)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Design r16; founder "return breakdown - approved"</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B48 finding 1 final wording: 'Everything you own and owe, in one place' + property examples (founder pick)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4062,6 +4062,33 @@
       <c r="E44" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>First-run setup</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>First bullet: "Everything you own and owe, in one place — accounts (investment, 401k, checking, savings), your home and other property, debts — one live view." (was "Map your whole money picture")</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>B48 walk finding 1 + founder second thought; matches the Net worth screen's Own − Owe language</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Founder (decision round)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B48 finding 1, final: 'All your assets and debts in one place' (founder wording)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4089,6 +4089,33 @@
       <c r="E45" t="inlineStr">
         <is>
           <t>Founder (decision round)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>First-run setup</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>First bullet FINAL: "All your assets and debts in one place" (founder's own wording, superseding the same-day own-and-owe pick)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>B48 walk finding 1, round 3</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B48 finding 1 CLOSED: parallel-examples bullet (founder: 'love it')
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4116,6 +4116,33 @@
       <c r="E46" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>First-run setup</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>First bullet CLOSED: "All your assets and debts in one place — accounts (investment, 401k, checking, savings), your home and other property, and every debt (mortgage, cards, loans) — one live view."</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>B48 finding 1 final round — complete-inventory principle + parallel examples</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Founder ("love it")</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase-1 simplification: PE/HF capture chips removed (founder); kinds stay in the data model
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4143,6 +4143,33 @@
       <c r="E47" t="inlineStr">
         <is>
           <t>Founder ("love it")</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Alternatives capture</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Private equity + Hedge funds OUT of phase 1 (founder: keep it simple) — capture chips trimmed on both editors; data model keeps the kinds so anything saved still renders</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Founder decision</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tab rename: Invest -> Performance (founder: 'Net worth · Performance'); one TAB_META change + copy sweep + pins; route keys unchanged
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4170,6 +4170,33 @@
       <c r="E48" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Navigation (all surfaces)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>The Invest tab is renamed PERFORMANCE (founder pick: Net worth · Performance) — one TAB_META change sweeps the bottom bar, menu strip, and desktop sidebar; tab-name copy swept on 3 screens. Route keys unchanged.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Two tabs kept; names now say what-I-have vs how-it's-doing</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Founder (decision)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pair v6: By-type removed (founder); two pills — By category / By institution; decision logged
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4197,6 +4197,33 @@
       <c r="E49" t="inlineStr">
         <is>
           <t>Founder (decision)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Net worth</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>BY TYPE view REMOVED (founder — resolves the open By-type question); WHAT YOU OWN restructures to the three uber-categories (Cash / Investments / Personal property) with classes as rows inside; two grouping pills remain: By category · By institution. Investments total = Performance total by definition (sweep cash under Cash).</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Pair-mock rounds v2-v6</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pair v7: 'Your retirement plan' row title (founder wording); logged
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4222,6 +4222,33 @@
         </is>
       </c>
       <c r="E50" t="inlineStr">
+        <is>
+          <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Net worth</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>"Your path ahead (from your Plan)" renamed "Your retirement plan" (founder wording)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Pair-mock round v7</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
         </is>

</xml_diff>

<commit_message>
Approved retirement words BUILT: onCourseSentence helper (workers lead with pot-at-retirement, retirees with lasting; refused below 80%), Plan hub wired, 4 pins, v14 mock, changelog row 52
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4251,6 +4251,33 @@
       <c r="E51" t="inlineStr">
         <is>
           <t>Founder (chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Plan (hub) + Net worth</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Retirement verdict wording: working = "Likely — retire at {65} with ~{pot at retirement}, lasting past {92} with ~{leftover} to spare"; retired = "Holding — on course to last past {92}, ~{leftover} to spare". Sentence only shown at 80%+ chance; numbers = median of the same simulation the odds use (never re-derived). Replaces "on course for ~$890,000 by 92".</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Founder read "by 92" as "working till 92" — ambiguous; workers act on the retirement-day pot first, survival second. 92 = plan-to age, 65 = retirement age: both dials now named in the sentence.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Founder ("approve these words", chat 2026-08-04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Banded sections on ALL FIVE tab screens (NW/Performance/Cashflow join Home/Plan) — 24 bands total via one SectionBand; suite 1400 green; web export green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4357,6 +4357,33 @@
         </is>
       </c>
       <c r="E55" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>All five tabs</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Banded sections BUILT on the five tab screens (Home 4 · Plan 6 · Net worth 5 · Performance 3 · Cash flow 6 bands) via the ONE SectionBand component; totals ride the bands; capture-surface sections use the light sub-band. Detail screens (~25) queued next.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Founder order: apply the adopted band pattern to all screens.</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
         </is>

</xml_diff>

<commit_message>
FOUNDER RULE: NW change % measured on cash + investments (denominator named on the line); invDaily capture beside nwDaily; never back-guessed; helper + 10 pins; mock v20; changelog row
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4384,6 +4384,33 @@
         </is>
       </c>
       <c r="E56" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Net worth</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>NW change PERCENT re-based onto cash + investments (denominator named on the line: "+0.5% on cash + investments"); dollar change stays full NW. Store now captures a daily cash+investments point (invDaily) beside the nw point; percent shows only once that history exists — never back-guessed. Helper investableChangePct pinned (8 tests) + 2 screen pins.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Founder: "calculating NW % on total is not meaningful — property increments are hand-captured." Percent must measure money that actually moves daily.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
         </is>

</xml_diff>

<commit_message>
Changelog row 59: value-walk structure approved for both walks (net-worth wording + debt-principal line confirmed by founder)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4440,6 +4440,33 @@
       <c r="E58" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Net worth + Performance</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Value-walk structure APPROVED for both walks: Beginning value → ＋Contributions → −Withdrawals → WEALTH GENERATED (light sub-band; rows: Dividends · Interest · Change in investment value) → Ending value. Founder-confirmed calls: NW sheet says "net worth" (home+debts have no market feed) and carries the extra "＋ Debt principal you paid" line so the walk always sums; Performance uses the exact "market value" labels. Mocks: networth-final-v6 (sheet) + performance-final-v2 (walk card).</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>One walk grammar everywhere; rows must sum exactly to the ending value.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Founder ("agree with both", chat 2026-08-04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pin the depth-sentence scoping rule (silent on short windows, speaks on year-scale figures); changelog row
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4494,6 +4494,33 @@
       <c r="E60" t="inlineStr">
         <is>
           <t>Founder ("makes sense. Let's do it.", chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Net worth (change sheet + banner)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Scoping rule for the depth sentence: it appears ONLY where the figure's window predates the source's shared history (12-month income yes; a 1-day change line no) — otherwise it implies older income sits inside the change number. Pinned. Walk sheet: all numbers share one right edge (WEALTH GENERATED total included); ＋ signs dropped, − kept. Mock networth-final-v8.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Founder: the history line "should only appear if the since-date is older than the shared history — otherwise the user thinks older dividends are added to the change number."</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CONSISTENCY SWEEP (founder order): 622 font sizes snapped to the one design scale across 70 files, white/grey hardcodes -> theme tokens in 42 files, 2 guard tests pin both rules; suite 1419 green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4519,6 +4519,33 @@
         </is>
       </c>
       <c r="E61" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>All screens</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>CONSISTENCY SWEEP: every fontSize snapped to the ONE design scale (11/13/15/17/20/24/30/38 — ties rounded UP for 55-70 readability): 622 values across 70 files. Hardcoded white/#F5F5F5 replaced with theme tokens in 42 files. Two guard tests added so drift cannot return.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Founder: "make sure font size and color and overall design are same across all screens."</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
         </is>

</xml_diff>

<commit_message>
NW FINAL built: uber-groups + donut back on screen (masked, 44pt legend) + Own-Owe above hero (duplicate line removed) + two pills only; finding-14 re-pinned; 1423 green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4546,6 +4546,33 @@
         </is>
       </c>
       <c r="E62" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Net worth</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>FINAL design BUILT (part 1): three uber-groups (Cash · Investments · Personal property) as collapsible light-green bars carrying totals, with asset classes as rows inside; class donut returned to the screen (validated palette, direct-labeled legend, 44pt targets, masks with hide-balances); Own − Owe moved ABOVE the hero and the duplicate bottom math line removed; pills trimmed to two (By category · By institution — By type removed). Finding-14 cash-merge rule re-pinned on the class view.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Founder: "build all the approved NW".</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
         </is>

</xml_diff>

<commit_message>
NW final: missing-data banner + fix-it sheet built on a new dataGaps engine (5 checks, inline never pop-up, fix buttons land on the exact cure); 8 pins; 1431 green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4573,6 +4573,33 @@
         </is>
       </c>
       <c r="E63" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Net worth (+ engine)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>MISSING-DATA BANNER + FIX-IT SHEET BUILT: new dataGaps engine (5 checks — unpriced holding · stale connection · no dividend records · stale hand-entered value · shared-history depth) feeding an INLINE banner (never a pop-up) that counts and names each gap; tapping opens the sheet where each row states what is missing, what we do meanwhile, and a button landing on the exact cure. Renders nothing when data is complete. 7 engine pins + 1 screen pin.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Founder disclaimer rule: say nothing when complete; speak only when a promised number is missing an input.</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
         </is>

</xml_diff>

<commit_message>
NW FINAL COMPLETE: change-tap walk sheet + buildChangeWalk engine (rows sum to ending by construction, net-worth wording, debt-principal line); 4 pins; 1435 green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4600,6 +4600,33 @@
         </is>
       </c>
       <c r="E64" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Net worth (change tap)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CHANGE WALK SHEET BUILT (final mock State E): tapping the change opens the walk in the approved structure — Beginning net worth → Contributions → Withdrawals → Wealth generated (Dividends · Interest · Change in investment value) → Debt principal you paid → Ending net worth. buildChangeWalk engine makes the rows sum to the ending value by construction (residual lands in change-in-value, never dropped). 3 engine pins + 1 screen pin. NET-WORTH FINAL IS NOW COMPLETE: 6 of 6 approved elements built.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Founder-approved walk structure + "design it exactly as the Performance walk card".</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
         </is>

</xml_diff>

<commit_message>
Performance final part 1: summary trio + value walk (approved order, rows sum by construction) + banner below summary; legacy breakdown block removed; tests re-pinned; 1435 green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4627,6 +4627,33 @@
         </is>
       </c>
       <c r="E65" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>FINAL design part 1 BUILT: SUMMARY trio (ending value · wealth generated · return) with the plain window sentence ("for the window you picked — not a yearly rate; money you added never counts as return"); the VALUE WALK card in the approved order (beginning market value → contributions → withdrawals → wealth generated (dividends · interest · change in investment value) → ending market value), rows summing by construction via buildChangeWalk; missing-data banner below the summary. The old inline return-breakdown block was REMOVED — superseded by the walk (one concept, one place). One periodStartKey definition now feeds the walk, the ledger filter and the gap checks.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Founder final Performance spec + banner-below-summary instruction.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
         </is>

</xml_diff>

<commit_message>
Performance final part 2 + account page: chips carry returns, category-earnings table, holdings under class sub-bands with per-holding income, all record doors per class; 1439 green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4654,6 +4654,33 @@
         </is>
       </c>
       <c r="E66" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Performance + Account page</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>FINAL design part 2 BUILT: period chips carry their OWN window return (em-dash when a window has no data, row wraps to two lines); category-earnings table (CATEGORY | EARNED | RETURN, ledger-only, absent entirely when nothing was received). ACCOUNT PAGE restructured to the final mock: holdings grouped under their CLASS on the light-green sub-band ("BY CATEGORY &amp; HOLDING"), each holding carrying its own income line beneath it (income belongs to the holding that earned it), and every kind of record has a door — money in/out, income received, buy/sale — tightened per class (property keeps none; cash gains an interest door it never had).</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Founder final Performance spec incl. "income below individual asset", "class sub-bands", "missing button to add sales/buy transaction".</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
         </is>

</xml_diff>

<commit_message>
Performance COMPLETE: per-account collapsible walks (one engine, parts sum to the whole); NW-family sub-screens banded; 1440 green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4683,6 +4683,33 @@
       <c r="E67" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Performance + NW family</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>PERFORMANCE COMPLETE: per-account collapsible walks added (same engine as the all-accounts walk; collapsed by default with a one-line wealth-generated summary, expanding to the full walk; hidden when only one account exists). NW-family sub-screens banded (Import holdings, Bonds &amp; CDs, Alternatives, SnapTrade connect). 7 of 7 Performance elements and 6 of 6 Net-worth elements now built.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Founder: "complete fully building NW and perf section".</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build 50 walk sheet + the release row in the changelog
32 rows in the order you would tap them, each saying what you do and what you should see, with your
Pass/Fail and comment columns. The five checks a test cannot make are marked Device-only — largest
text size, reduce motion, a grayscale look at both bars, app-switcher masking, and the keyboard over
a save button on the smallest phone.

A second tab records what is in the build, what is knowingly still open, and the one thing verified
by nothing but your eyes: how the dated banner title wraps at the largest text size.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5059,6 +5059,33 @@
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>BUILD 50 CUT (v1.1.0 build 50, from commit 8e09374 on taxonomy-v1.0.7) after the founder's explicit "cut the build" to a presented pre-build checklist. Gate satisfied in order: scope complete (59 of 59 tracker rows), audits FINISHED (mock-match audit round 1+2, and the 9-row open-gaps ledger re-verified against the live code and closed with the test that pins each), adversarial journey pass green (4 suites / 64 tests), then the checklist. Fresh gates at the cut: 1,492 tests green, tsc clean, UI-test gate passing, clean tree. Contents: the Net worth Quiet-Instrument rebuild, the founder's 11 hero corrections, his 6 audit decisions, the dated hero title, the one-banner titling, and 6 defects found during the audit (2 dead routes among them). Walk sheet: docs/FCC-core-55-70/build50-founder-walk-2026-08-11.xlsx.</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Founder: "cut the build" (2026-08-11), replying to the pre-build checklist.</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-11)</t>
         </is>

</xml_diff>